<commit_message>
Add step 4 with sending report to slack
</commit_message>
<xml_diff>
--- a/src/test/resources/data/TestResults.xlsx
+++ b/src/test/resources/data/TestResults.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="25">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="82" uniqueCount="25">
   <si>
     <t>STT</t>
   </si>
@@ -162,10 +162,10 @@
         <v>6</v>
       </c>
       <c r="D2" t="s" s="0">
-        <v>8</v>
+        <v>14</v>
       </c>
       <c r="E2" t="s" s="0">
-        <v>13</v>
+        <v>15</v>
       </c>
     </row>
     <row r="3">
@@ -196,10 +196,10 @@
         <v>17</v>
       </c>
       <c r="D4" t="s" s="0">
-        <v>8</v>
+        <v>14</v>
       </c>
       <c r="E4" t="s" s="0">
-        <v>13</v>
+        <v>15</v>
       </c>
     </row>
     <row r="5">
@@ -213,10 +213,10 @@
         <v>20</v>
       </c>
       <c r="D5" t="s" s="0">
-        <v>21</v>
+        <v>14</v>
       </c>
       <c r="E5" t="s" s="0">
-        <v>22</v>
+        <v>15</v>
       </c>
     </row>
     <row r="6">

</xml_diff>

<commit_message>
n8n and update CI pipeline
</commit_message>
<xml_diff>
--- a/src/test/resources/data/TestResults.xlsx
+++ b/src/test/resources/data/TestResults.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="82" uniqueCount="25">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="92" uniqueCount="25">
   <si>
     <t>STT</t>
   </si>
@@ -179,10 +179,10 @@
         <v>11</v>
       </c>
       <c r="D3" t="s" s="0">
-        <v>14</v>
+        <v>8</v>
       </c>
       <c r="E3" t="s" s="0">
-        <v>15</v>
+        <v>13</v>
       </c>
     </row>
     <row r="4">

</xml_diff>